<commit_message>
fix(squad1): Serra Grande passa para a Aura Minerals na carteira de projetos
GO-008 (Mina Crixás / Serra Grande) estava atribuída à AngloGold Ashanti.
A AngloGold anunciou a venda da Mineração Serra Grande à Aura Minerals em
02/06/2025, e a Aura informou o fechamento da aquisição em 01/12/2025,
como já registra producao/base_curada.json.

Na planilha do Lucas Maia: empresa e controladora passam a Aura Minerals,
a data da informação vai para 01/12/2025, e a transação entra em "Outras
evidências" e "Links adicionais". A evidência principal e a produção de
80.000 oz/ano ficam como estavam, porque são do relatório de 2024 da
AngloGold, e as observações dizem isso. Pacote do Mercado regenerado.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Squad 1/Dados brutos/Aluno Lucas Maia/projetos_minerais_goias.xlsx
+++ b/Squad 1/Dados brutos/Aluno Lucas Maia/projetos_minerais_goias.xlsx
@@ -1699,12 +1699,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AngloGold Ashanti</t>
+          <t>Aura Minerals</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>AngloGold Ashanti plc</t>
+          <t>Aura Minerals Inc.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1804,7 +1804,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2024-02-15</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
@@ -1829,17 +1829,17 @@
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>Venda anunciada pela AngloGold Ashanti em 02/06/2025; fechamento da aquisição informado pela Aura em 01/12/2025</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>https://www.auraminerals.com/investors/</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>Uma das frentes operacionais de ouro mais longevas do Brasil, com expansão constante de frentes subterrâneas profundas.</t>
+          <t>Uma das frentes operacionais de ouro mais longevas do Brasil, com expansão constante de frentes subterrâneas profundas. Operada pela AngloGold Ashanti até 11/2025; desde 01/12/2025 pertence à Aura Minerals. A evidência principal e a produção de 80.000 oz/ano são do período AngloGold (relatório de 2024).</t>
         </is>
       </c>
     </row>

</xml_diff>